<commit_message>
refactor!: rename subracer to subhound
Rename the package, CLI, runtime identifiers, documentation, and tests.

Expand gitignore rules for local environments, caches, editors, and secrets.
</commit_message>
<xml_diff>
--- a/tests/reports/identify_report.xlsx
+++ b/tests/reports/identify_report.xlsx
@@ -454,7 +454,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>subracer identify() report</t>
+          <t>subhound identify() report</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-17 21:40:50</t>
+          <t>2026-06-21 21:05:21</t>
         </is>
       </c>
     </row>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="N82" s="5" t="inlineStr">
         <is>
-          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: subracer/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_01/The X-Files (1993)/s01/Fallen_Angel.mkv</t>
+          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: SubHound/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_01/The X-Files (1993)/s01/Fallen_Angel.mkv</t>
         </is>
       </c>
     </row>
@@ -6149,7 +6149,7 @@
       </c>
       <c r="N102" s="5" t="inlineStr">
         <is>
-          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: subracer/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_02/The X-Files (1993)/s1/Fallen_Angel.mkv</t>
+          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: SubHound/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_02/The X-Files (1993)/s1/Fallen_Angel.mkv</t>
         </is>
       </c>
     </row>
@@ -7271,7 +7271,7 @@
       </c>
       <c r="N122" s="5" t="inlineStr">
         <is>
-          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: subracer/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_03/The X-Files (1993)/season1/Fallen_Angel.mkv</t>
+          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: SubHound/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_03/The X-Files (1993)/season1/Fallen_Angel.mkv</t>
         </is>
       </c>
     </row>
@@ -8393,7 +8393,7 @@
       </c>
       <c r="N142" s="5" t="inlineStr">
         <is>
-          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: subracer/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_04/The X-Files (1993)/season_01/Fallen_Angel.mkv</t>
+          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: SubHound/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_04/The X-Files (1993)/season_01/Fallen_Angel.mkv</t>
         </is>
       </c>
     </row>
@@ -9515,7 +9515,7 @@
       </c>
       <c r="N162" s="5" t="inlineStr">
         <is>
-          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: subracer/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_05/The X-Files (1993)/season_1/Fallen_Angel.mkv</t>
+          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: SubHound/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_05/The X-Files (1993)/season_1/Fallen_Angel.mkv</t>
         </is>
       </c>
     </row>
@@ -10637,7 +10637,7 @@
       </c>
       <c r="N182" s="5" t="inlineStr">
         <is>
-          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: subracer/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_06/The X-Files (1993)/S01/Fallen_Angel.mkv</t>
+          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: SubHound/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_06/The X-Files (1993)/S01/Fallen_Angel.mkv</t>
         </is>
       </c>
     </row>
@@ -11759,7 +11759,7 @@
       </c>
       <c r="N202" s="5" t="inlineStr">
         <is>
-          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: subracer/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_07/The X-Files (1993)/S1/Fallen_Angel.mkv</t>
+          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: SubHound/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_07/The X-Files (1993)/S1/Fallen_Angel.mkv</t>
         </is>
       </c>
     </row>
@@ -12881,7 +12881,7 @@
       </c>
       <c r="N222" s="5" t="inlineStr">
         <is>
-          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: subracer/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_08/The X-Files (1993)/Season 01/Fallen_Angel.mkv</t>
+          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: SubHound/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_08/The X-Files (1993)/Season 01/Fallen_Angel.mkv</t>
         </is>
       </c>
     </row>
@@ -14003,7 +14003,7 @@
       </c>
       <c r="N242" s="5" t="inlineStr">
         <is>
-          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: subracer/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_09/The X-Files (1993)/Season 1/Fallen_Angel.mkv</t>
+          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: SubHound/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_09/The X-Files (1993)/Season 1/Fallen_Angel.mkv</t>
         </is>
       </c>
     </row>
@@ -15125,7 +15125,7 @@
       </c>
       <c r="N262" s="5" t="inlineStr">
         <is>
-          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: subracer/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_10/The X-Files (1993)/season01/Fallen_Angel.mkv</t>
+          <t>TV show 'The X-Files' detected but the episode number could not be determined from filename or folders: SubHound/tests/data/portable_media_test_set/edge_cases/season_folder_filename_matrix/variant_10/The X-Files (1993)/season01/Fallen_Angel.mkv</t>
         </is>
       </c>
     </row>

</xml_diff>